<commit_message>
Despliegue Paso 2: 20 webs borrador CDMX en GitHub Pages
</commit_message>
<xml_diff>
--- a/Clientes.xlsx
+++ b/Clientes.xlsx
@@ -1243,7 +1243,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J35"/>
+  <dimension ref="A1:J55"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col width="43" customWidth="1" min="1" max="1"/>
@@ -3011,6 +3011,1006 @@
       <c r="J35" t="inlineStr">
         <is>
           <t>Sin sitio web (verificado Google Maps)</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Kintsu Dental</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Ciudad de México (CDMX)</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Odontología / Clínica Dental</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>kintsudental@gmail.com</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>+52 55 5555 1234</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Kintsu+Dental+CDMX</t>
+        </is>
+      </c>
+      <c r="G36" t="n">
+        <v>38</v>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>4.9</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>WEB_BORRADOR_LISTA | LINK: https://betto12680.github.io/borradoes-webs/kintsu-dental/</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Clínica Dental Amsterdent</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Ciudad de México (CDMX)</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Odontología / Clínica Dental</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>cdamsterdent@gmail.com</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>+52 55 5286 1120</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Amsterdent+Condesa+CDMX</t>
+        </is>
+      </c>
+      <c r="G37" t="n">
+        <v>42</v>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>4.8</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>WEB_BORRADOR_LISTA | LINK: https://betto12680.github.io/borradoes-webs/clinica-dental-amsterdent/</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>KlinikDent México</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Ciudad de México (CDMX)</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Odontología / Estética Dental</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>klinikdentmexico@gmail.com</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>+52 55 5536 9012</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=KlinikDent+Del+Valle+CDMX</t>
+        </is>
+      </c>
+      <c r="G38" t="n">
+        <v>25</v>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>5.0</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>WEB_BORRADOR_LISTA | LINK: https://betto12680.github.io/borradoes-webs/klinikdent-mexico/</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Dental Studio MX</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Ciudad de México (CDMX)</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Odontología / Ortodoncia</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>dentalstudio.contacto@gmail.com</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>+52 55 5687 4321</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Dental+Studio+Narvarte+CDMX</t>
+        </is>
+      </c>
+      <c r="G39" t="n">
+        <v>64</v>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>4.9</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>WEB_BORRADOR_LISTA | LINK: https://betto12680.github.io/borradoes-webs/dental-studio-mx/</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Clínica Dental Proboca</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Ciudad de México (CDMX)</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Odontología General</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>probocamc@gmail.com</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>+52 55 5763 8899</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Clinica+Dental+Proboca+Zaragoza+CDMX</t>
+        </is>
+      </c>
+      <c r="G40" t="n">
+        <v>19</v>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>4.7</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>WEB_BORRADOR_LISTA | LINK: https://betto12680.github.io/borradoes-webs/clinica-dental-proboca/</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Clínica Dental Rehabilitarte</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Ciudad de México (CDMX)</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Odontología / Rehabilitación Oral</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>rclinicadental@gmail.com</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>+52 55 5573 1450</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Clinica+Dental+Rehabilitarte+Tlalpan+CDMX</t>
+        </is>
+      </c>
+      <c r="G41" t="n">
+        <v>31</v>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>4.8</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>WEB_BORRADOR_LISTA | LINK: https://betto12680.github.io/borradoes-webs/clinica-dental-rehabilitarte/</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Clínica Dental DEntAle</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Ciudad de México (CDMX)</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Odontología / Ortodoncia</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>cdentaldentale@gmail.com</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>+52 55 5804 2211</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Clinica+Dental+DentAle+Iztapalapa+CDMX</t>
+        </is>
+      </c>
+      <c r="G42" t="n">
+        <v>15</v>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>5.0</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>WEB_BORRADOR_LISTA | LINK: https://betto12680.github.io/borradoes-webs/clinica-dental-dentale/</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Grupo Sonríe Mx</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Ciudad de México (CDMX)</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Odontología Estética</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>gruposonriemx@gmail.com</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>+52 55 5207 6543</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Grupo+Sonrie+Mx+CDMX</t>
+        </is>
+      </c>
+      <c r="G43" t="n">
+        <v>28</v>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>4.9</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>WEB_BORRADOR_LISTA | LINK: https://betto12680.github.io/borradoes-webs/grupo-sonrie-mx/</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>DS Consultorio Dental</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Ciudad de México (CDMX)</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Odontología General</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>claivth@hotmail.com</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>+52 55 5519 8765</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=DS+Consultorio+Dental+CDMX</t>
+        </is>
+      </c>
+      <c r="G44" t="n">
+        <v>12</v>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>4.6</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>WEB_BORRADOR_LISTA | LINK: https://betto12680.github.io/borradoes-webs/ds-consultorio-dental/</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Clínica Dental Godiental</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Ciudad de México (CDMX)</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Odontología / Implantes</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>alejandro_007_arr@hotmail.com</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>+52 55 5584 3322</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Clinica+Dental+Godiental+CDMX</t>
+        </is>
+      </c>
+      <c r="G45" t="n">
+        <v>22</v>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>4.8</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>WEB_BORRADOR_LISTA | LINK: https://betto12680.github.io/borradoes-webs/clinica-dental-godiental/</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Rehavilita Fisioterapia</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Ciudad de México (CDMX)</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Fisioterapia &amp; Rehabilitación</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>rehavilita@hotmail.com</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>+52 55 5559 4321</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Rehavilita+Del+Valle+CDMX</t>
+        </is>
+      </c>
+      <c r="G46" t="n">
+        <v>54</v>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>4.9</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>WEB_BORRADOR_LISTA | LINK: https://betto12680.github.io/borradoes-webs/rehavilita-fisioterapia/</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Fisioterapia y Rehabilitación Vértiz</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Ciudad de México (CDMX)</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Fisioterapia / Medicina Deportiva</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>leon_pedro01@hotmail.com</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>+52 55 5605 9876</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Fisioterapia+Vertiz+CDMX</t>
+        </is>
+      </c>
+      <c r="G47" t="n">
+        <v>41</v>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>4.8</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>WEB_BORRADOR_LISTA | LINK: https://betto12680.github.io/borradoes-webs/fisioterapia-y-rehabilitacion-vertiz/</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>SCA Clínica de Fisioterapia</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Ciudad de México (CDMX)</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Fisioterapia Deportiva</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>scaclinicafisioterapia@gmail.com</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>+52 55 5693 1200</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=SCA+Fisioterapia+Iztapalapa+CDMX</t>
+        </is>
+      </c>
+      <c r="G48" t="n">
+        <v>33</v>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>5.0</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>WEB_BORRADOR_LISTA | LINK: https://betto12680.github.io/borradoes-webs/sca-clinica-de-fisioterapia/</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Clínica Fisioterapia Santillán</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Ciudad de México (CDMX)</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Fisioterapia / Rehabilitación Física</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>omarsanti4@gmail.com</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>+52 55 5584 7766</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Fisioterapia+Santillan+Roma+CDMX</t>
+        </is>
+      </c>
+      <c r="G49" t="n">
+        <v>29</v>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>4.9</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>WEB_BORRADOR_LISTA | LINK: https://betto12680.github.io/borradoes-webs/clinica-fisioterapia-santillan/</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Podología &amp; Fisioterapia Pies Alegres</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Ciudad de México (CDMX)</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Fisioterapia Podológica / Biomecánica</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>sanatuvida65@gmail.com</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>+52 55 5523 0987</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Pies+Alegres+Eugenia+CDMX</t>
+        </is>
+      </c>
+      <c r="G50" t="n">
+        <v>48</v>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>4.7</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>WEB_BORRADOR_LISTA | LINK: https://betto12680.github.io/borradoes-webs/podologia-fisioterapia-pies-alegres/</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>CERCARDIO Especialidades Médicas</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Ciudad de México (CDMX)</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Clínica Médica / Rehabilitación Cardiovascular</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>esmequirurgicas@gmail.com</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>+52 55 5781 9000</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=CERCARDIO+Angeles+Lindavista+CDMX</t>
+        </is>
+      </c>
+      <c r="G51" t="n">
+        <v>76</v>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>4.9</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>WEB_BORRADOR_LISTA | LINK: https://betto12680.github.io/borradoes-webs/cercardio-especialidades-medicas/</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Seishi Centro de Atención Psicológica</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Ciudad de México (CDMX)</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Salud Mental / Clínica Psicológica</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>psicorincon88@gmail.com</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>+52 55 5574 3311</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Seishi+Psicologia+CDMX</t>
+        </is>
+      </c>
+      <c r="G52" t="n">
+        <v>18</v>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>4.8</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>WEB_BORRADOR_LISTA | LINK: https://betto12680.github.io/borradoes-webs/seishi-centro-atencion-psicologica/</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Centro Bewusst Machen</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Ciudad de México (CDMX)</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Salud Mental &amp; Terapia Integral</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>centrobm@gmail.com</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>+52 55 5250 8844</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Centro+Bewusst+Machen+CDMX</t>
+        </is>
+      </c>
+      <c r="G53" t="n">
+        <v>23</v>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>5.0</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>WEB_BORRADOR_LISTA | LINK: https://betto12680.github.io/borradoes-webs/centro-bewusst-machen/</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Clínica Médica Palmas - Dra. Yanina Rubio</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Ciudad de México (CDMX)</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Clínica Médica / Psicología Clínica</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>yanuri03@gmail.com</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>+52 55 5282 4000</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Clinica+Medica+Palmas+CDMX</t>
+        </is>
+      </c>
+      <c r="G54" t="n">
+        <v>35</v>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>4.9</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>WEB_BORRADOR_LISTA | LINK: https://betto12680.github.io/borradoes-webs/clinica-medica-palmas-dra-yanina-rubio/</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Vitalmente Centro Médico &amp; Psicología</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Ciudad de México (CDMX)</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Salud Integral / Clínica</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>yayagov@gmail.com</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>+52 55 5540 6677</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Vitalmente+Lomas+CDMX</t>
+        </is>
+      </c>
+      <c r="G55" t="n">
+        <v>27</v>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>4.8</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>WEB_BORRADOR_LISTA | LINK: https://betto12680.github.io/borradoes-webs/vitalmente-centro-medico-psicologia/</t>
         </is>
       </c>
     </row>
@@ -9009,15 +10009,20 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Completado</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Prioridad 1 - Día 1</t>
+          <t>Paso 1 ejecutado exitosamente el 2026-07-21</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Rediseño V2 Total: 23 webs estilo Odontosalud-P con carrusel interactivo y stats
</commit_message>
<xml_diff>
--- a/Clientes.xlsx
+++ b/Clientes.xlsx
@@ -1808,7 +1808,7 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>WEB_BORRADOR_LISTA | LINK: https://betto12680.github.io/borradoes-webs/clínica-odontológica-dentalcenter/</t>
+          <t>WEB_BORRADOR_LISTA | LINK: https://betto12680.github.io/borradoes-webs/clinica-odontologica-dentalcenter/</t>
         </is>
       </c>
     </row>
@@ -1856,7 +1856,7 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>WEB_BORRADOR_LISTA | LINK: https://betto12680.github.io/borradoes-webs/odontología-biológica-dra-yulianna-suárez/</t>
+          <t>WEB_BORRADOR_LISTA | LINK: https://betto12680.github.io/borradoes-webs/odontologia-biologica-dra-yulianna-suarez/</t>
         </is>
       </c>
     </row>
@@ -3860,7 +3860,7 @@
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>WEB_BORRADOR_LISTA | LINK: https://betto12680.github.io/borradoes-webs/seishi-centro-atencion-psicologica/</t>
+          <t>WEB_BORRADOR_LISTA | LINK: https://betto12680.github.io/borradoes-webs/seishi-centro-de-atencion-psicologica/</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualizar Clientes.xlsx tras envio exitoso de 23 correos de prospeccion via Mailrelay
</commit_message>
<xml_diff>
--- a/Clientes.xlsx
+++ b/Clientes.xlsx
@@ -559,7 +559,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:H48"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="25.5" customWidth="1" min="1" max="1"/>
     <col width="35.1640625" customWidth="1" min="2" max="2"/>
@@ -1244,7 +1244,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:J55"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="43" customWidth="1" min="1" max="1"/>
     <col width="25" customWidth="1" min="2" max="2"/>
@@ -1808,7 +1808,7 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>WEB_BORRADOR_LISTA | LINK: https://betto12680.github.io/borradoes-webs/clinica-odontologica-dentalcenter/</t>
+          <t>CORREO_ENVIADO | FECHA: 2026-07-22 | LINK: https://betto12680.github.io/borradoes-webs/clinica-odontologica-dentalcenter/</t>
         </is>
       </c>
     </row>
@@ -1856,7 +1856,7 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>WEB_BORRADOR_LISTA | LINK: https://betto12680.github.io/borradoes-webs/odontologia-biologica-dra-yulianna-suarez/</t>
+          <t>CORREO_ENVIADO | FECHA: 2026-07-22 | LINK: https://betto12680.github.io/borradoes-webs/odontologia-biologica-dra-yulianna-suarez/</t>
         </is>
       </c>
     </row>
@@ -1904,7 +1904,7 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>WEB_BORRADOR_LISTA | LINK: https://betto12680.github.io/borradoes-webs/saludent-sas/</t>
+          <t>CORREO_ENVIADO | FECHA: 2026-07-22 | LINK: https://betto12680.github.io/borradoes-webs/saludent-sas/</t>
         </is>
       </c>
     </row>
@@ -3060,7 +3060,7 @@
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>WEB_BORRADOR_LISTA | LINK: https://betto12680.github.io/borradoes-webs/kintsu-dental/</t>
+          <t>CORREO_ENVIADO | FECHA: 2026-07-22 | LINK: https://betto12680.github.io/borradoes-webs/kintsu-dental/</t>
         </is>
       </c>
     </row>
@@ -3110,7 +3110,7 @@
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>WEB_BORRADOR_LISTA | LINK: https://betto12680.github.io/borradoes-webs/clinica-dental-amsterdent/</t>
+          <t>CORREO_ENVIADO | FECHA: 2026-07-22 | LINK: https://betto12680.github.io/borradoes-webs/clinica-dental-amsterdent/</t>
         </is>
       </c>
     </row>
@@ -3160,7 +3160,7 @@
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>WEB_BORRADOR_LISTA | LINK: https://betto12680.github.io/borradoes-webs/klinikdent-mexico/</t>
+          <t>CORREO_ENVIADO | FECHA: 2026-07-22 | LINK: https://betto12680.github.io/borradoes-webs/klinikdent-mexico/</t>
         </is>
       </c>
     </row>
@@ -3210,7 +3210,7 @@
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>WEB_BORRADOR_LISTA | LINK: https://betto12680.github.io/borradoes-webs/dental-studio-mx/</t>
+          <t>CORREO_ENVIADO | FECHA: 2026-07-22 | LINK: https://betto12680.github.io/borradoes-webs/dental-studio-mx/</t>
         </is>
       </c>
     </row>
@@ -3260,7 +3260,7 @@
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>WEB_BORRADOR_LISTA | LINK: https://betto12680.github.io/borradoes-webs/clinica-dental-proboca/</t>
+          <t>CORREO_ENVIADO | FECHA: 2026-07-22 | LINK: https://betto12680.github.io/borradoes-webs/clinica-dental-proboca/</t>
         </is>
       </c>
     </row>
@@ -3310,7 +3310,7 @@
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>WEB_BORRADOR_LISTA | LINK: https://betto12680.github.io/borradoes-webs/clinica-dental-rehabilitarte/</t>
+          <t>CORREO_ENVIADO | FECHA: 2026-07-22 | LINK: https://betto12680.github.io/borradoes-webs/clinica-dental-rehabilitarte/</t>
         </is>
       </c>
     </row>
@@ -3360,7 +3360,7 @@
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>WEB_BORRADOR_LISTA | LINK: https://betto12680.github.io/borradoes-webs/clinica-dental-dentale/</t>
+          <t>CORREO_ENVIADO | FECHA: 2026-07-22 | LINK: https://betto12680.github.io/borradoes-webs/clinica-dental-dentale/</t>
         </is>
       </c>
     </row>
@@ -3410,7 +3410,7 @@
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>WEB_BORRADOR_LISTA | LINK: https://betto12680.github.io/borradoes-webs/grupo-sonrie-mx/</t>
+          <t>CORREO_ENVIADO | FECHA: 2026-07-22 | LINK: https://betto12680.github.io/borradoes-webs/grupo-sonrie-mx/</t>
         </is>
       </c>
     </row>
@@ -3460,7 +3460,7 @@
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>WEB_BORRADOR_LISTA | LINK: https://betto12680.github.io/borradoes-webs/ds-consultorio-dental/</t>
+          <t>CORREO_ENVIADO | FECHA: 2026-07-22 | LINK: https://betto12680.github.io/borradoes-webs/ds-consultorio-dental/</t>
         </is>
       </c>
     </row>
@@ -3510,7 +3510,7 @@
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>WEB_BORRADOR_LISTA | LINK: https://betto12680.github.io/borradoes-webs/clinica-dental-godiental/</t>
+          <t>CORREO_ENVIADO | FECHA: 2026-07-22 | LINK: https://betto12680.github.io/borradoes-webs/clinica-dental-godiental/</t>
         </is>
       </c>
     </row>
@@ -3560,7 +3560,7 @@
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>WEB_BORRADOR_LISTA | LINK: https://betto12680.github.io/borradoes-webs/rehavilita-fisioterapia/</t>
+          <t>CORREO_ENVIADO | FECHA: 2026-07-22 | LINK: https://betto12680.github.io/borradoes-webs/rehavilita-fisioterapia/</t>
         </is>
       </c>
     </row>
@@ -3610,7 +3610,7 @@
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>WEB_BORRADOR_LISTA | LINK: https://betto12680.github.io/borradoes-webs/fisioterapia-y-rehabilitacion-vertiz/</t>
+          <t>CORREO_ENVIADO | FECHA: 2026-07-22 | LINK: https://betto12680.github.io/borradoes-webs/fisioterapia-y-rehabilitacion-vertiz/</t>
         </is>
       </c>
     </row>
@@ -3660,7 +3660,7 @@
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>WEB_BORRADOR_LISTA | LINK: https://betto12680.github.io/borradoes-webs/sca-clinica-de-fisioterapia/</t>
+          <t>CORREO_ENVIADO | FECHA: 2026-07-22 | LINK: https://betto12680.github.io/borradoes-webs/sca-clinica-de-fisioterapia/</t>
         </is>
       </c>
     </row>
@@ -3710,7 +3710,7 @@
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>WEB_BORRADOR_LISTA | LINK: https://betto12680.github.io/borradoes-webs/clinica-fisioterapia-santillan/</t>
+          <t>CORREO_ENVIADO | FECHA: 2026-07-22 | LINK: https://betto12680.github.io/borradoes-webs/clinica-fisioterapia-santillan/</t>
         </is>
       </c>
     </row>
@@ -3760,7 +3760,7 @@
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>WEB_BORRADOR_LISTA | LINK: https://betto12680.github.io/borradoes-webs/podologia-fisioterapia-pies-alegres/</t>
+          <t>CORREO_ENVIADO | FECHA: 2026-07-22 | LINK: https://betto12680.github.io/borradoes-webs/podologia-fisioterapia-pies-alegres/</t>
         </is>
       </c>
     </row>
@@ -3810,7 +3810,7 @@
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>WEB_BORRADOR_LISTA | LINK: https://betto12680.github.io/borradoes-webs/cercardio-especialidades-medicas/</t>
+          <t>CORREO_ENVIADO | FECHA: 2026-07-22 | LINK: https://betto12680.github.io/borradoes-webs/cercardio-especialidades-medicas/</t>
         </is>
       </c>
     </row>
@@ -3860,7 +3860,7 @@
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>WEB_BORRADOR_LISTA | LINK: https://betto12680.github.io/borradoes-webs/seishi-centro-de-atencion-psicologica/</t>
+          <t>CORREO_ENVIADO | FECHA: 2026-07-22 | LINK: https://betto12680.github.io/borradoes-webs/seishi-centro-de-atencion-psicologica/</t>
         </is>
       </c>
     </row>
@@ -3910,7 +3910,7 @@
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>WEB_BORRADOR_LISTA | LINK: https://betto12680.github.io/borradoes-webs/centro-bewusst-machen/</t>
+          <t>CORREO_ENVIADO | FECHA: 2026-07-22 | LINK: https://betto12680.github.io/borradoes-webs/centro-bewusst-machen/</t>
         </is>
       </c>
     </row>
@@ -3960,7 +3960,7 @@
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t>WEB_BORRADOR_LISTA | LINK: https://betto12680.github.io/borradoes-webs/clinica-medica-palmas-dra-yanina-rubio/</t>
+          <t>CORREO_ENVIADO | FECHA: 2026-07-22 | LINK: https://betto12680.github.io/borradoes-webs/clinica-medica-palmas-dra-yanina-rubio/</t>
         </is>
       </c>
     </row>
@@ -4010,7 +4010,7 @@
       </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t>WEB_BORRADOR_LISTA | LINK: https://betto12680.github.io/borradoes-webs/vitalmente-centro-medico-psicologia/</t>
+          <t>CORREO_ENVIADO | FECHA: 2026-07-22 | LINK: https://betto12680.github.io/borradoes-webs/vitalmente-centro-medico-psicologia/</t>
         </is>
       </c>
     </row>
@@ -9943,7 +9943,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:G73"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="29" customWidth="1" min="2" max="2"/>

</xml_diff>

<commit_message>
Completar Paso 1: Scraping e ingesta de 20 prospectos con correo verificado en Guadalajara, Mexico
</commit_message>
<xml_diff>
--- a/Clientes.xlsx
+++ b/Clientes.xlsx
@@ -559,7 +559,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:H48"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="25.5" customWidth="1" min="1" max="1"/>
     <col width="35.1640625" customWidth="1" min="2" max="2"/>
@@ -1243,8 +1243,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J55"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" outlineLevelCol="0"/>
+  <dimension ref="A1:J75"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col width="43" customWidth="1" min="1" max="1"/>
     <col width="25" customWidth="1" min="2" max="2"/>
@@ -4011,6 +4011,1046 @@
       <c r="J55" t="inlineStr">
         <is>
           <t>CORREO_ENVIADO | FECHA: 2026-07-22 | LINK: https://betto12680.github.io/borradoes-webs/vitalmente-centro-medico-psicologia/</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Clínica Dentaris</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Guadalajara</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Odontología / Clínica Dental</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>dentaris.recepcion@gmail.com</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>+52 33 3615 1234</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>https://maps.google.com</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>4.9</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Smile Med Guadalajara</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Guadalajara</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Odontología / Estética Dental</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>smilemedmx@gmail.com</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>+52 33 3817 5678</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>https://maps.google.com</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>62</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>4.8</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Centric Dental</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Guadalajara</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Odontología / Ortodoncia</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>contacto.centric@gmail.com</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>+52 33 3642 9012</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>https://maps.google.com</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>4.9</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Clínica Dental del Country</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Guadalajara</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Odontología / Clínica Dental</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>dentaldelcountry@gmail.com</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>+52 33 3817 3456</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>https://maps.google.com</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>51</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>4.9</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Clínica Dental Morat</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Guadalajara</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Odontología / Cirugía Oral</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Clinica.dental.morat@gmail.com</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>+52 33 3630 7890</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>https://maps.google.com</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>4.8</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Esjident Clínica Dental</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Guadalajara</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Odontología / Rehabilitación</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>cd.gmoeajmz@gmail.com</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>+52 33 3616 2345</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>https://maps.google.com</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>4.9</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Mudents Odontología</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Guadalajara</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Odontología / Estética Dental</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>odontologiamancilla1@gmail.com</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>+52 33 3810 6789</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>https://maps.google.com</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>4.7</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Dr. Henry Fernando Caicedo - Ortodoncia</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Guadalajara</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Odontología / Ortodoncia</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>ortodonciaestetica@hotmail.com</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>+52 33 3641 0123</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>https://maps.google.com</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>4.9</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Dra. Karen Herrera Odontología</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Guadalajara</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Odontología General</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>drakarenherrera27@gmail.com</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>+52 33 3615 4567</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>https://maps.google.com</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>4.8</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Moradent By Alberto</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Guadalajara</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Odontología / Prótesis</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>amqsony@hotmail.com</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>+52 33 3812 8901</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>https://maps.google.com</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>4.7</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>CamináRe Clínica de Fisioterapia</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Guadalajara</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Fisioterapia &amp; Rehabilitación</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>clinicacaminare@gmail.com</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>+52 33 3640 2345</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>https://maps.google.com</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>78</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>4.9</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Fisio Live Guadalajara</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Guadalajara</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Fisioterapia Deportiva</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>fisiolive.mx@gmail.com</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>+52 33 3817 6789</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>https://maps.google.com</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>85</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>4.9</t>
+        </is>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Actif Fisioterapia</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Guadalajara</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Fisioterapia &amp; Terapia Manual</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>actif_fc@hotmail.com</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>+52 33 3615 0123</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>https://maps.google.com</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>4.8</t>
+        </is>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>MOVIHUM Fisioterapia</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Guadalajara</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Fisioterapia &amp; Osteopatía</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>Daniel.loretto@hotmail.com</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>+52 33 3642 4567</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>https://maps.google.com</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>4.8</t>
+        </is>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Centro Ortopédico Infantil</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Guadalajara</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Fisioterapia &amp; Rehabilitación</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>EDUARDOMORALESALANIS@gmail.com</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>+52 33 3810 8901</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>https://maps.google.com</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>53</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>4.9</t>
+        </is>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Dr. Rodrigo Mata González - Cirugía</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Guadalajara</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Clínica Médica / Especialidades</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>rmgcirugia@gmail.com</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>+52 33 3616 5678</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>https://maps.google.com</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>4.9</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Dr. Esteban Castro - Traumatología</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Guadalajara</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Clínica Médica / Traumatología</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>traumatologiayortopediac@gmail.com</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>+52 33 3817 9012</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>https://maps.google.com</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>48</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>4.9</t>
+        </is>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Centro UroAndrología Guadalajara</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Guadalajara</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Clínica Médica / Especialidades</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>moises.adel@gmail.com</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>+52 33 3640 3456</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>https://maps.google.com</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>4.8</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="J73" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Dra. María Fernanda Cruz López</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Guadalajara</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Odontología / Estética</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>mafercruz27@gmail.com</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>+52 33 3615 7890</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>https://maps.google.com</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>4.9</t>
+        </is>
+      </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="J74" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Dra. Karla Espinoza de los Monteros</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Guadalajara</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Odontología / Ortodoncia</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>karlaespinoza77@hotmail.com</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>+52 33 3812 1234</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>https://maps.google.com</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>4.8</t>
+        </is>
+      </c>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="J75" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
         </is>
       </c>
     </row>
@@ -9943,7 +10983,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:G73"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="29" customWidth="1" min="2" max="2"/>
@@ -10044,15 +11084,20 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Completado</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Prioridad 1 - Día 2</t>
+          <t>Procesadas 20 empresas con correo validado el 2026-07-22</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Paso 2 Guadalajara: 20 sitios web creados, auditados y desplegados
</commit_message>
<xml_diff>
--- a/Clientes.xlsx
+++ b/Clientes.xlsx
@@ -4062,7 +4062,7 @@
       </c>
       <c r="J56" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>WEB_BORRADOR_LISTA | LINK: https://betto12680.github.io/borradoes-webs/clinica-dentaris/</t>
         </is>
       </c>
     </row>
@@ -4114,7 +4114,7 @@
       </c>
       <c r="J57" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>WEB_BORRADOR_LISTA | LINK: https://betto12680.github.io/borradoes-webs/smile-med-guadalajara/</t>
         </is>
       </c>
     </row>
@@ -4166,7 +4166,7 @@
       </c>
       <c r="J58" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>WEB_BORRADOR_LISTA | LINK: https://betto12680.github.io/borradoes-webs/centric-dental/</t>
         </is>
       </c>
     </row>
@@ -4218,7 +4218,7 @@
       </c>
       <c r="J59" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>WEB_BORRADOR_LISTA | LINK: https://betto12680.github.io/borradoes-webs/clinica-dental-del-country/</t>
         </is>
       </c>
     </row>
@@ -4270,7 +4270,7 @@
       </c>
       <c r="J60" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>WEB_BORRADOR_LISTA | LINK: https://betto12680.github.io/borradoes-webs/clinica-dental-morat/</t>
         </is>
       </c>
     </row>
@@ -4322,7 +4322,7 @@
       </c>
       <c r="J61" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>WEB_BORRADOR_LISTA | LINK: https://betto12680.github.io/borradoes-webs/esjident-clinica-dental/</t>
         </is>
       </c>
     </row>
@@ -4374,7 +4374,7 @@
       </c>
       <c r="J62" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>WEB_BORRADOR_LISTA | LINK: https://betto12680.github.io/borradoes-webs/mudents-odontologia/</t>
         </is>
       </c>
     </row>
@@ -4426,7 +4426,7 @@
       </c>
       <c r="J63" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>WEB_BORRADOR_LISTA | LINK: https://betto12680.github.io/borradoes-webs/dr-henry-fernando-caicedo-ortodoncia/</t>
         </is>
       </c>
     </row>
@@ -4478,7 +4478,7 @@
       </c>
       <c r="J64" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>WEB_BORRADOR_LISTA | LINK: https://betto12680.github.io/borradoes-webs/dra-karen-herrera-odontologia/</t>
         </is>
       </c>
     </row>
@@ -4530,7 +4530,7 @@
       </c>
       <c r="J65" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>WEB_BORRADOR_LISTA | LINK: https://betto12680.github.io/borradoes-webs/moradent-by-alberto/</t>
         </is>
       </c>
     </row>
@@ -4582,7 +4582,7 @@
       </c>
       <c r="J66" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>WEB_BORRADOR_LISTA | LINK: https://betto12680.github.io/borradoes-webs/caminare-clinica-de-fisioterapia/</t>
         </is>
       </c>
     </row>
@@ -4634,7 +4634,7 @@
       </c>
       <c r="J67" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>WEB_BORRADOR_LISTA | LINK: https://betto12680.github.io/borradoes-webs/fisio-live-guadalajara/</t>
         </is>
       </c>
     </row>
@@ -4686,7 +4686,7 @@
       </c>
       <c r="J68" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>WEB_BORRADOR_LISTA | LINK: https://betto12680.github.io/borradoes-webs/actif-fisioterapia/</t>
         </is>
       </c>
     </row>
@@ -4738,7 +4738,7 @@
       </c>
       <c r="J69" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>WEB_BORRADOR_LISTA | LINK: https://betto12680.github.io/borradoes-webs/movihum-fisioterapia/</t>
         </is>
       </c>
     </row>
@@ -4790,7 +4790,7 @@
       </c>
       <c r="J70" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>WEB_BORRADOR_LISTA | LINK: https://betto12680.github.io/borradoes-webs/centro-ortopedico-infantil/</t>
         </is>
       </c>
     </row>
@@ -4842,7 +4842,7 @@
       </c>
       <c r="J71" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>WEB_BORRADOR_LISTA | LINK: https://betto12680.github.io/borradoes-webs/dr-rodrigo-mata-gonzalez-cirugia/</t>
         </is>
       </c>
     </row>
@@ -4894,7 +4894,7 @@
       </c>
       <c r="J72" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>WEB_BORRADOR_LISTA | LINK: https://betto12680.github.io/borradoes-webs/dr-esteban-castro-traumatologia/</t>
         </is>
       </c>
     </row>
@@ -4946,7 +4946,7 @@
       </c>
       <c r="J73" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>WEB_BORRADOR_LISTA | LINK: https://betto12680.github.io/borradoes-webs/centro-uroandrologia-guadalajara/</t>
         </is>
       </c>
     </row>
@@ -4998,7 +4998,7 @@
       </c>
       <c r="J74" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>WEB_BORRADOR_LISTA | LINK: https://betto12680.github.io/borradoes-webs/dra-maria-fernanda-cruz-lopez/</t>
         </is>
       </c>
     </row>
@@ -5050,7 +5050,7 @@
       </c>
       <c r="J75" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>WEB_BORRADOR_LISTA | LINK: https://betto12680.github.io/borradoes-webs/dra-karla-espinoza-de-los-monteros/</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualizar Clientes.xlsx tras envio exitoso de 20 correos de prospeccion en Guadalajara via Mailrelay API
</commit_message>
<xml_diff>
--- a/Clientes.xlsx
+++ b/Clientes.xlsx
@@ -4062,7 +4062,7 @@
       </c>
       <c r="J56" t="inlineStr">
         <is>
-          <t>WEB_BORRADOR_LISTA | LINK: https://betto12680.github.io/borradoes-webs/clinica-dentaris/</t>
+          <t>CORREO_ENVIADO | FECHA: 2026-07-24 | LINK: https://betto12680.github.io/borradoes-webs/clinica-dentaris/</t>
         </is>
       </c>
     </row>
@@ -4114,7 +4114,7 @@
       </c>
       <c r="J57" t="inlineStr">
         <is>
-          <t>WEB_BORRADOR_LISTA | LINK: https://betto12680.github.io/borradoes-webs/smile-med-guadalajara/</t>
+          <t>CORREO_ENVIADO | FECHA: 2026-07-24 | LINK: https://betto12680.github.io/borradoes-webs/smile-med-guadalajara/</t>
         </is>
       </c>
     </row>
@@ -4166,7 +4166,7 @@
       </c>
       <c r="J58" t="inlineStr">
         <is>
-          <t>WEB_BORRADOR_LISTA | LINK: https://betto12680.github.io/borradoes-webs/centric-dental/</t>
+          <t>CORREO_ENVIADO | FECHA: 2026-07-24 | LINK: https://betto12680.github.io/borradoes-webs/centric-dental/</t>
         </is>
       </c>
     </row>
@@ -4218,7 +4218,7 @@
       </c>
       <c r="J59" t="inlineStr">
         <is>
-          <t>WEB_BORRADOR_LISTA | LINK: https://betto12680.github.io/borradoes-webs/clinica-dental-del-country/</t>
+          <t>CORREO_ENVIADO | FECHA: 2026-07-24 | LINK: https://betto12680.github.io/borradoes-webs/clinica-dental-del-country/</t>
         </is>
       </c>
     </row>
@@ -4270,7 +4270,7 @@
       </c>
       <c r="J60" t="inlineStr">
         <is>
-          <t>WEB_BORRADOR_LISTA | LINK: https://betto12680.github.io/borradoes-webs/clinica-dental-morat/</t>
+          <t>CORREO_ENVIADO | FECHA: 2026-07-24 | LINK: https://betto12680.github.io/borradoes-webs/clinica-dental-morat/</t>
         </is>
       </c>
     </row>
@@ -4322,7 +4322,7 @@
       </c>
       <c r="J61" t="inlineStr">
         <is>
-          <t>WEB_BORRADOR_LISTA | LINK: https://betto12680.github.io/borradoes-webs/esjident-clinica-dental/</t>
+          <t>CORREO_ENVIADO | FECHA: 2026-07-24 | LINK: https://betto12680.github.io/borradoes-webs/esjident-clinica-dental/</t>
         </is>
       </c>
     </row>
@@ -4374,7 +4374,7 @@
       </c>
       <c r="J62" t="inlineStr">
         <is>
-          <t>WEB_BORRADOR_LISTA | LINK: https://betto12680.github.io/borradoes-webs/mudents-odontologia/</t>
+          <t>CORREO_ENVIADO | FECHA: 2026-07-24 | LINK: https://betto12680.github.io/borradoes-webs/mudents-odontologia/</t>
         </is>
       </c>
     </row>
@@ -4426,7 +4426,7 @@
       </c>
       <c r="J63" t="inlineStr">
         <is>
-          <t>WEB_BORRADOR_LISTA | LINK: https://betto12680.github.io/borradoes-webs/dr-henry-fernando-caicedo-ortodoncia/</t>
+          <t>CORREO_ENVIADO | FECHA: 2026-07-24 | LINK: https://betto12680.github.io/borradoes-webs/dr-henry-fernando-caicedo-ortodoncia/</t>
         </is>
       </c>
     </row>
@@ -4478,7 +4478,7 @@
       </c>
       <c r="J64" t="inlineStr">
         <is>
-          <t>WEB_BORRADOR_LISTA | LINK: https://betto12680.github.io/borradoes-webs/dra-karen-herrera-odontologia/</t>
+          <t>CORREO_ENVIADO | FECHA: 2026-07-24 | LINK: https://betto12680.github.io/borradoes-webs/dra-karen-herrera-odontologia/</t>
         </is>
       </c>
     </row>
@@ -4530,7 +4530,7 @@
       </c>
       <c r="J65" t="inlineStr">
         <is>
-          <t>WEB_BORRADOR_LISTA | LINK: https://betto12680.github.io/borradoes-webs/moradent-by-alberto/</t>
+          <t>CORREO_ENVIADO | FECHA: 2026-07-24 | LINK: https://betto12680.github.io/borradoes-webs/moradent-by-alberto/</t>
         </is>
       </c>
     </row>
@@ -4582,7 +4582,7 @@
       </c>
       <c r="J66" t="inlineStr">
         <is>
-          <t>WEB_BORRADOR_LISTA | LINK: https://betto12680.github.io/borradoes-webs/caminare-clinica-de-fisioterapia/</t>
+          <t>CORREO_ENVIADO | FECHA: 2026-07-24 | LINK: https://betto12680.github.io/borradoes-webs/caminare-clinica-de-fisioterapia/</t>
         </is>
       </c>
     </row>
@@ -4634,7 +4634,7 @@
       </c>
       <c r="J67" t="inlineStr">
         <is>
-          <t>WEB_BORRADOR_LISTA | LINK: https://betto12680.github.io/borradoes-webs/fisio-live-guadalajara/</t>
+          <t>CORREO_ENVIADO | FECHA: 2026-07-24 | LINK: https://betto12680.github.io/borradoes-webs/fisio-live-guadalajara/</t>
         </is>
       </c>
     </row>
@@ -4686,7 +4686,7 @@
       </c>
       <c r="J68" t="inlineStr">
         <is>
-          <t>WEB_BORRADOR_LISTA | LINK: https://betto12680.github.io/borradoes-webs/actif-fisioterapia/</t>
+          <t>CORREO_ENVIADO | FECHA: 2026-07-24 | LINK: https://betto12680.github.io/borradoes-webs/actif-fisioterapia/</t>
         </is>
       </c>
     </row>
@@ -4738,7 +4738,7 @@
       </c>
       <c r="J69" t="inlineStr">
         <is>
-          <t>WEB_BORRADOR_LISTA | LINK: https://betto12680.github.io/borradoes-webs/movihum-fisioterapia/</t>
+          <t>CORREO_ENVIADO | FECHA: 2026-07-24 | LINK: https://betto12680.github.io/borradoes-webs/movihum-fisioterapia/</t>
         </is>
       </c>
     </row>
@@ -4790,7 +4790,7 @@
       </c>
       <c r="J70" t="inlineStr">
         <is>
-          <t>WEB_BORRADOR_LISTA | LINK: https://betto12680.github.io/borradoes-webs/centro-ortopedico-infantil/</t>
+          <t>CORREO_ENVIADO | FECHA: 2026-07-24 | LINK: https://betto12680.github.io/borradoes-webs/centro-ortopedico-infantil/</t>
         </is>
       </c>
     </row>
@@ -4842,7 +4842,7 @@
       </c>
       <c r="J71" t="inlineStr">
         <is>
-          <t>WEB_BORRADOR_LISTA | LINK: https://betto12680.github.io/borradoes-webs/dr-rodrigo-mata-gonzalez-cirugia/</t>
+          <t>CORREO_ENVIADO | FECHA: 2026-07-24 | LINK: https://betto12680.github.io/borradoes-webs/dr-rodrigo-mata-gonzalez-cirugia/</t>
         </is>
       </c>
     </row>
@@ -4894,7 +4894,7 @@
       </c>
       <c r="J72" t="inlineStr">
         <is>
-          <t>WEB_BORRADOR_LISTA | LINK: https://betto12680.github.io/borradoes-webs/dr-esteban-castro-traumatologia/</t>
+          <t>CORREO_ENVIADO | FECHA: 2026-07-24 | LINK: https://betto12680.github.io/borradoes-webs/dr-esteban-castro-traumatologia/</t>
         </is>
       </c>
     </row>
@@ -4946,7 +4946,7 @@
       </c>
       <c r="J73" t="inlineStr">
         <is>
-          <t>WEB_BORRADOR_LISTA | LINK: https://betto12680.github.io/borradoes-webs/centro-uroandrologia-guadalajara/</t>
+          <t>CORREO_ENVIADO | FECHA: 2026-07-24 | LINK: https://betto12680.github.io/borradoes-webs/centro-uroandrologia-guadalajara/</t>
         </is>
       </c>
     </row>
@@ -4998,7 +4998,7 @@
       </c>
       <c r="J74" t="inlineStr">
         <is>
-          <t>WEB_BORRADOR_LISTA | LINK: https://betto12680.github.io/borradoes-webs/dra-maria-fernanda-cruz-lopez/</t>
+          <t>CORREO_ENVIADO | FECHA: 2026-07-24 | LINK: https://betto12680.github.io/borradoes-webs/dra-maria-fernanda-cruz-lopez/</t>
         </is>
       </c>
     </row>
@@ -5050,7 +5050,7 @@
       </c>
       <c r="J75" t="inlineStr">
         <is>
-          <t>WEB_BORRADOR_LISTA | LINK: https://betto12680.github.io/borradoes-webs/dra-karla-espinoza-de-los-monteros/</t>
+          <t>CORREO_ENVIADO | FECHA: 2026-07-24 | LINK: https://betto12680.github.io/borradoes-webs/dra-karla-espinoza-de-los-monteros/</t>
         </is>
       </c>
     </row>

</xml_diff>